<commit_message>
Update fixture metadata for new data representation
- Add gdp_component column to transactions sheet in ta_classifications.xlsx
- Add columns.xlsx: two-column column/role mapping for SUTColumns

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/ta_classifications.xlsx
+++ b/data/fixtures/metadata/ta_classifications.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,6 +580,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>gdp_component</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -592,6 +597,11 @@
           <t>Output at basic prices</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -604,6 +614,11 @@
           <t>Imports</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>imports</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -616,6 +631,11 @@
           <t>Intermediate consumption</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -628,6 +648,11 @@
           <t>Household consumption</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>private_consumption</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -640,6 +665,11 @@
           <t>Government collective consumption</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>government_consumption</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -652,6 +682,11 @@
           <t>Gross fixed capital formation - dwellings</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>investment</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -662,6 +697,11 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Exports of domestic production</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>exports</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename classification column description -> name
The 'description' label implied a note or prose explanation.
'name' better reflects the intent: the official standard text
name for a code (product, transaction, industry, consumption function).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/ta_classifications.xlsx
+++ b/data/fixtures/metadata/ta_classifications.xlsx
@@ -515,7 +515,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>name</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove gdp_component from SUTClassifications and metadata format
GDP decomposition mapping is analysis-time input, not SUT metadata.
Rationale: chaining and aggregation do not commute — GDP must be computed
at the right aggregation level before chaining. Valid gdp_component values
are settled and documented for future use as a function argument.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/ta_classifications.xlsx
+++ b/data/fixtures/metadata/ta_classifications.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,11 +580,6 @@
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>gdp_component</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -597,11 +592,6 @@
           <t>Output at basic prices</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>output</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -614,11 +604,6 @@
           <t>Imports</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>imports</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -631,11 +616,6 @@
           <t>Intermediate consumption</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>intermediate</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -648,11 +628,6 @@
           <t>Household consumption</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>private_consumption</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -665,11 +640,6 @@
           <t>Government collective consumption</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>government_consumption</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -682,11 +652,6 @@
           <t>Gross fixed capital formation - dwellings</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>investment</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -697,11 +662,6 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Exports of domestic production</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>exports</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement metadata loaders and update fixtures
- sutlab/io.py: implement load_metadata_columns_from_excel,
  load_metadata_classifications_from_excel, load_metadata_from_excel.
  Validates roles, required columns, table values; strips whitespace;
  reads all values as strings.
- tests/test_io.py: 36 tests covering happy paths, whitespace stripping,
  integer column names, all error cases.
- data/fixtures/generate.py: add table column (supply/use) to transactions.
- data/fixtures/metadata/ta_classifications.xlsx: regenerated with table column.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/ta_classifications.xlsx
+++ b/data/fixtures/metadata/ta_classifications.xlsx
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,6 +580,11 @@
           <t>name</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -592,6 +597,11 @@
           <t>Output at basic prices</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>supply</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -604,6 +614,11 @@
           <t>Imports</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>supply</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -616,6 +631,11 @@
           <t>Intermediate consumption</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -628,6 +648,11 @@
           <t>Household consumption</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -640,6 +665,11 @@
           <t>Government collective consumption</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -652,6 +682,11 @@
           <t>Gross fixed capital formation - dwellings</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>use</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -662,6 +697,11 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Exports of domestic production</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>use</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add esa_code to transactions and split category code lookup by type
Adds required esa_code column to the transactions classification sheet,
mapping institution-specific codes to standardised ESA codes (P1, P2,
P31, P32, etc.). Replaces get_category_codes with three specific functions:
get_industry_codes (P1/P2), get_individual_consumption_codes (P31), and
get_collective_consumption_codes (P32).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fixtures/metadata/ta_classifications.xlsx
+++ b/data/fixtures/metadata/ta_classifications.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,6 +597,11 @@
           <t>table</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>esa_code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -614,6 +619,11 @@
           <t>supply</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -631,6 +641,11 @@
           <t>supply</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -648,6 +663,11 @@
           <t>use</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -665,6 +685,11 @@
           <t>use</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>P31</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -682,6 +707,11 @@
           <t>use</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>P32</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -699,6 +729,11 @@
           <t>use</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>P51g</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -716,6 +751,11 @@
           <t>use</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>P52</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -731,6 +771,11 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>use</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>P6</t>
         </is>
       </c>
     </row>

</xml_diff>